<commit_message>
fix: PKSF Fashion Garments lab list 11 -> 22 items
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYF8ZViZ52j72cGLCGYpbD
</commit_message>
<xml_diff>
--- a/data/xlsx/pksf--fashion-garments.xlsx
+++ b/data/xlsx/pksf--fashion-garments.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
@@ -132,6 +132,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -497,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.17" customWidth="1" min="1" max="1"/>
@@ -637,12 +643,12 @@
       </c>
     </row>
     <row r="16" ht="14.15" customHeight="1">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="14" t="n">
         <v>1</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Computers/Laptop</t>
+          <t>Computer/ Laptop</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
@@ -661,12 +667,12 @@
       <c r="G16" s="9" t="n"/>
     </row>
     <row r="17" ht="14.15" customHeight="1">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="14" t="n">
         <v>2</v>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Projector &amp; Screen (HD quality, HDMI support, 3000+ lumens)</t>
+          <t>Multimedia Projector</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
@@ -676,7 +682,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F17" s="9">
         <f>IFERROR(MIN(C17,D17)*E17/C17,0)</f>
@@ -685,22 +691,22 @@
       <c r="G17" s="9" t="n"/>
     </row>
     <row r="18" ht="14.15" customHeight="1">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="14" t="n">
         <v>3</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Printer</t>
+          <t>Table for Printing</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F18" s="9">
         <f>IFERROR(MIN(C18,D18)*E18/C18,0)</f>
@@ -709,12 +715,12 @@
       <c r="G18" s="9" t="n"/>
     </row>
     <row r="19" ht="14.15" customHeight="1">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="14" t="n">
         <v>4</v>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Mannequins/Dress Forms (Female and male standard sizes)</t>
+          <t>Fabric Cutting Table</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
@@ -724,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F19" s="9">
         <f>IFERROR(MIN(C19,D19)*E19/C19,0)</f>
@@ -733,16 +739,16 @@
       <c r="G19" s="9" t="n"/>
     </row>
     <row r="20" ht="14.15" customHeight="1">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="14" t="n">
         <v>5</v>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Single needle lock stitch machine</t>
+          <t>Pattern Making Table</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D20" s="9" t="n">
         <v>0</v>
@@ -757,22 +763,22 @@
       <c r="G20" s="9" t="n"/>
     </row>
     <row r="21" ht="14.15" customHeight="1">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="14" t="n">
         <v>6</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Overlock machine</t>
+          <t>Mannequin doll (Child, male and female)</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F21" s="9">
         <f>IFERROR(MIN(C21,D21)*E21/C21,0)</f>
@@ -781,22 +787,22 @@
       <c r="G21" s="9" t="n"/>
     </row>
     <row r="22" ht="14.15" customHeight="1">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="14" t="n">
         <v>7</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Cutting table (60”x 50”)</t>
+          <t>Sample Fashion Garments Product</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D22" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F22" s="9">
         <f>IFERROR(MIN(C22,D22)*E22/C22,0)</f>
@@ -805,22 +811,22 @@
       <c r="G22" s="9" t="n"/>
     </row>
     <row r="23" ht="14.15" customHeight="1">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="14" t="n">
         <v>8</v>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Electric iron</t>
+          <t>Sample Technical Package</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F23" s="9">
         <f>IFERROR(MIN(C23,D23)*E23/C23,0)</f>
@@ -829,22 +835,22 @@
       <c r="G23" s="9" t="n"/>
     </row>
     <row r="24" ht="14.15" customHeight="1">
-      <c r="A24" s="7" t="n">
+      <c r="A24" s="14" t="n">
         <v>9</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Electric steam iron with iron table</t>
+          <t>Sample Motif and Embellishment</t>
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F24" s="9">
         <f>IFERROR(MIN(C24,D24)*E24/C24,0)</f>
@@ -853,12 +859,12 @@
       <c r="G24" s="9" t="n"/>
     </row>
     <row r="25" ht="14.15" customHeight="1">
-      <c r="A25" s="7" t="n">
+      <c r="A25" s="14" t="n">
         <v>10</v>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Scissors (10”-12”)</t>
+          <t>Sets of Pattern Making Curves</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
@@ -868,7 +874,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F25" s="9">
         <f>IFERROR(MIN(C25,D25)*E25/C25,0)</f>
@@ -877,12 +883,12 @@
       <c r="G25" s="9" t="n"/>
     </row>
     <row r="26" ht="14.15" customHeight="1">
-      <c r="A26" s="7" t="n">
+      <c r="A26" s="14" t="n">
         <v>11</v>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Sewing tool box</t>
+          <t>Tracing Wheels</t>
         </is>
       </c>
       <c r="C26" s="9" t="n">
@@ -892,7 +898,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F26" s="9">
         <f>IFERROR(MIN(C26,D26)*E26/C26,0)</f>
@@ -900,57 +906,321 @@
       </c>
       <c r="G26" s="9" t="n"/>
     </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+    <row r="27" ht="14.15" customHeight="1">
+      <c r="A27" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Hoops and Frames Set</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" s="9">
+        <f>IFERROR(MIN(C27,D27)*E27/C27,0)</f>
+        <v/>
+      </c>
+      <c r="G27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="14.15" customHeight="1">
+      <c r="A28" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Embroidery Machine</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F28" s="9">
+        <f>IFERROR(MIN(C28,D28)*E28/C28,0)</f>
+        <v/>
+      </c>
+      <c r="G28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="14.15" customHeight="1">
+      <c r="A29" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Different Dices for Block for Printing</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" s="9">
+        <f>IFERROR(MIN(C29,D29)*E29/C29,0)</f>
+        <v/>
+      </c>
+      <c r="G29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="14.15" customHeight="1">
+      <c r="A30" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Different Screen for Printing</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" s="9">
+        <f>IFERROR(MIN(C30,D30)*E30/C30,0)</f>
+        <v/>
+      </c>
+      <c r="G30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="14.15" customHeight="1">
+      <c r="A31" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Burner for Dyeing and Printing</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F31" s="9">
+        <f>IFERROR(MIN(C31,D31)*E31/C31,0)</f>
+        <v/>
+      </c>
+      <c r="G31" s="9" t="n"/>
+    </row>
+    <row r="32" ht="14.15" customHeight="1">
+      <c r="A32" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Fabric Cutting Scissor (6-10 inches)</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F32" s="9">
+        <f>IFERROR(MIN(C32,D32)*E32/C32,0)</f>
+        <v/>
+      </c>
+      <c r="G32" s="9" t="n"/>
+    </row>
+    <row r="33" ht="14.15" customHeight="1">
+      <c r="A33" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Straight Knife</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" s="9">
+        <f>IFERROR(MIN(C33,D33)*E33/C33,0)</f>
+        <v/>
+      </c>
+      <c r="G33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="14.15" customHeight="1">
+      <c r="A34" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Single Needle Machine (Domestic)</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F34" s="9">
+        <f>IFERROR(MIN(C34,D34)*E34/C34,0)</f>
+        <v/>
+      </c>
+      <c r="G34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="14.15" customHeight="1">
+      <c r="A35" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Single Needle Machine (Industrial)</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F35" s="9">
+        <f>IFERROR(MIN(C35,D35)*E35/C35,0)</f>
+        <v/>
+      </c>
+      <c r="G35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="14.15" customHeight="1">
+      <c r="A36" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Overlock Machines</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F36" s="9">
+        <f>IFERROR(MIN(C36,D36)*E36/C36,0)</f>
+        <v/>
+      </c>
+      <c r="G36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="14.15" customHeight="1">
+      <c r="A37" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Industrial Iron with Table</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F37" s="9">
+        <f>IFERROR(MIN(C37,D37)*E37/C37,0)</f>
+        <v/>
+      </c>
+      <c r="G37" s="9" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Sum</t>
         </is>
       </c>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="10">
-        <f>SUM(E16:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="10">
-        <f>SUM(F16:F26)</f>
-        <v/>
-      </c>
-      <c r="G27" s="13" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="11" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="15">
+        <f>SUM(E16:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="15">
+        <f>SUM(F16:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="13" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>Score out of 100</t>
         </is>
       </c>
-      <c r="B28" s="11" t="n"/>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="11" t="n"/>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="10">
-        <f>F27/E27*100</f>
-        <v/>
-      </c>
-      <c r="G28" s="13" t="n"/>
-    </row>
-    <row r="29" ht="9.75" customHeight="1"/>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="15">
+        <f>F38/E38*100</f>
+        <v/>
+      </c>
+      <c r="G39" s="13" t="n"/>
+    </row>
+    <row r="40" ht="9.75" customHeight="1"/>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Total achieved points out of 30  </t>
         </is>
       </c>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="10">
-        <f>F28*30/100</f>
-        <v/>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="15">
+        <f>F39*30/100</f>
+        <v/>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
@@ -958,13 +1228,13 @@
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A30:E30"/>
     <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A27:D27"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A41:E41"/>
     <mergeCell ref="C8:G8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>